<commit_message>
Updated YBLTE site metadata
</commit_message>
<xml_diff>
--- a/Data/tabular/YBLTE_sites.xlsx
+++ b/Data/tabular/YBLTE_sites.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eholmes\Box\Yolo_Food_Web\Data\tabular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECEB5395-145B-4DE9-8D4E-CD7FCC487E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4708A31-EE9A-4120-B5C0-C1419222FF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="65">
   <si>
     <t>Rowid</t>
   </si>
@@ -219,6 +219,18 @@
   </si>
   <si>
     <t>LEBLS ramp 1</t>
+  </si>
+  <si>
+    <t>LIS</t>
+  </si>
+  <si>
+    <t>Toe Drain at Lisbon Weir</t>
+  </si>
+  <si>
+    <t>Tide's end wetland drain canal</t>
+  </si>
+  <si>
+    <t>TEW-Drain</t>
   </si>
 </sst>
 </file>
@@ -260,7 +272,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -288,56 +300,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFFFCD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFD5D5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -623,9 +585,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="3" max="3" width="18.36328125" customWidth="1"/>
     <col min="4" max="4" width="36.7265625" customWidth="1"/>
     <col min="10" max="11" width="12.1796875" customWidth="1"/>
   </cols>
@@ -872,10 +835,10 @@
         <v>15</v>
       </c>
       <c r="J7">
-        <v>38.706180000000003</v>
+        <v>38.706584999999997</v>
       </c>
       <c r="K7">
-        <v>-121.64306999999999</v>
+        <v>-121.641075</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
@@ -906,6 +869,12 @@
       <c r="I8" t="s">
         <v>16</v>
       </c>
+      <c r="J8">
+        <v>38.706121000000003</v>
+      </c>
+      <c r="K8">
+        <v>-121.640055</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9">
@@ -935,6 +904,12 @@
       <c r="I9" t="s">
         <v>16</v>
       </c>
+      <c r="J9">
+        <v>38.706980999999999</v>
+      </c>
+      <c r="K9">
+        <v>-121.639974</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10">
@@ -964,6 +939,12 @@
       <c r="I10" t="s">
         <v>16</v>
       </c>
+      <c r="J10">
+        <v>38.678443999999999</v>
+      </c>
+      <c r="K10">
+        <v>-121.672147</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11">
@@ -994,10 +975,10 @@
         <v>16</v>
       </c>
       <c r="J11">
-        <v>38.676789999999997</v>
+        <v>38.675984999999997</v>
       </c>
       <c r="K11">
-        <v>-121.644233</v>
+        <v>-121.64358</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
@@ -1028,6 +1009,12 @@
       <c r="I12" t="s">
         <v>15</v>
       </c>
+      <c r="J12">
+        <v>38.647534999999998</v>
+      </c>
+      <c r="K12">
+        <v>-121.655367</v>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13">
@@ -1046,7 +1033,7 @@
         <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>16</v>
+        <v>58</v>
       </c>
       <c r="G13" t="s">
         <v>16</v>
@@ -1056,6 +1043,12 @@
       </c>
       <c r="I13" t="s">
         <v>16</v>
+      </c>
+      <c r="J13">
+        <v>38.668295999999998</v>
+      </c>
+      <c r="K13">
+        <v>-121.63758900000001</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
@@ -1122,10 +1115,10 @@
         <v>15</v>
       </c>
       <c r="J15">
-        <v>38.608150000000002</v>
+        <v>38.607045999999997</v>
       </c>
       <c r="K15">
-        <v>-121.571201</v>
+        <v>-121.572649</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
@@ -1145,7 +1138,7 @@
         <v>14</v>
       </c>
       <c r="F16" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="G16" t="s">
         <v>58</v>
@@ -1156,6 +1149,12 @@
       <c r="I16" t="s">
         <v>16</v>
       </c>
+      <c r="J16">
+        <v>38.607087999999997</v>
+      </c>
+      <c r="K16">
+        <v>-121.587768</v>
+      </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17">
@@ -1184,6 +1183,12 @@
       </c>
       <c r="I17" t="s">
         <v>15</v>
+      </c>
+      <c r="J17">
+        <v>38.573303000000003</v>
+      </c>
+      <c r="K17">
+        <v>-121.582909</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
@@ -1215,10 +1220,10 @@
         <v>16</v>
       </c>
       <c r="J18">
-        <v>38.574233999999997</v>
+        <v>38.550862000000002</v>
       </c>
       <c r="K18">
-        <v>-121.582543</v>
+        <v>-121.58289499999999</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
@@ -1229,13 +1234,13 @@
         <v>28</v>
       </c>
       <c r="C19" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="D19" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="E19" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F19" t="s">
         <v>15</v>
@@ -1244,16 +1249,16 @@
         <v>15</v>
       </c>
       <c r="H19" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="I19" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J19">
-        <v>38.400039999999997</v>
+        <v>38.476303000000001</v>
       </c>
       <c r="K19">
-        <v>-121.627999</v>
+        <v>-121.58860199999999</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
@@ -1264,13 +1269,13 @@
         <v>28</v>
       </c>
       <c r="C20" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E20" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F20" t="s">
         <v>15</v>
@@ -1285,24 +1290,21 @@
         <v>15</v>
       </c>
       <c r="J20">
-        <v>38.407192000000002</v>
+        <v>38.389926000000003</v>
       </c>
       <c r="K20">
-        <v>-121.62603900000001</v>
+        <v>-121.628434</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A21">
-        <v>20</v>
-      </c>
       <c r="B21" t="s">
         <v>28</v>
       </c>
       <c r="C21" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="D21" t="s">
-        <v>33</v>
+        <v>63</v>
       </c>
       <c r="E21" t="s">
         <v>14</v>
@@ -1311,7 +1313,7 @@
         <v>15</v>
       </c>
       <c r="G21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H21" t="s">
         <v>15</v>
@@ -1320,14 +1322,84 @@
         <v>16</v>
       </c>
       <c r="J21">
+        <v>38.390438000000003</v>
+      </c>
+      <c r="K21">
+        <v>-121.626563</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" t="s">
+        <v>15</v>
+      </c>
+      <c r="J22">
+        <v>38.418415000000003</v>
+      </c>
+      <c r="K22">
+        <v>-121.615256</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" t="s">
+        <v>16</v>
+      </c>
+      <c r="J23">
         <v>38.353357000000003</v>
       </c>
-      <c r="K21">
+      <c r="K23">
         <v>-121.643249</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:I21">
+  <conditionalFormatting sqref="F2:I23">
     <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="p">
       <formula>NOT(ISERROR(SEARCH("p",F2)))</formula>
     </cfRule>

</xml_diff>

<commit_message>
point wq QC + fish list/sorting code
</commit_message>
<xml_diff>
--- a/Data/tabular/YBLTE_sites.xlsx
+++ b/Data/tabular/YBLTE_sites.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eholmes\Box\Yolo_Food_Web\Data\tabular\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kristinn\Downloads\coding\YBLTE\Data\tabular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4708A31-EE9A-4120-B5C0-C1419222FF4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7CDA84F-9515-4122-BEF0-573665C9EABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15360" windowHeight="10800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="69">
   <si>
     <t>Rowid</t>
   </si>
@@ -119,9 +119,6 @@
     <t>Conaway Ranch</t>
   </si>
   <si>
-    <t>Above Lisbon Beach Seine site</t>
-  </si>
-  <si>
     <t>Lower</t>
   </si>
   <si>
@@ -161,9 +158,6 @@
     <t>LEBLS ramp 4 and lower terrace</t>
   </si>
   <si>
-    <t>FWALT</t>
-  </si>
-  <si>
     <t>I80</t>
   </si>
   <si>
@@ -231,6 +225,24 @@
   </si>
   <si>
     <t>TEW-Drain</t>
+  </si>
+  <si>
+    <t>BL5</t>
+  </si>
+  <si>
+    <t>Below Lisbon Beach Seine site</t>
+  </si>
+  <si>
+    <t>FW_Alt</t>
+  </si>
+  <si>
+    <t>AL1</t>
+  </si>
+  <si>
+    <t>Above Lisbon Beach Seine site 1</t>
+  </si>
+  <si>
+    <t>Above Lisbon Beach Seine site 0</t>
   </si>
 </sst>
 </file>
@@ -272,7 +284,127 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="15">
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFD5D5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFCD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFD5D5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFCD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFD5D5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFCD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFD5D5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFCD"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -585,15 +717,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="18.36328125" customWidth="1"/>
-    <col min="4" max="4" width="36.7265625" customWidth="1"/>
-    <col min="10" max="11" width="12.1796875" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="4" max="4" width="36.7109375" customWidth="1"/>
+    <col min="10" max="11" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -628,10 +760,10 @@
         <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -666,7 +798,7 @@
         <v>-121.63614099999999</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -701,7 +833,7 @@
         <v>-121.635724</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -709,10 +841,10 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E4" t="s">
         <v>19</v>
@@ -736,7 +868,7 @@
         <v>-121.636802</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -744,10 +876,10 @@
         <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E5" t="s">
         <v>14</v>
@@ -771,7 +903,7 @@
         <v>-121.634705</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -779,10 +911,10 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
@@ -791,7 +923,7 @@
         <v>15</v>
       </c>
       <c r="G6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H6" t="s">
         <v>16</v>
@@ -806,7 +938,7 @@
         <v>-121.66362700000001</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -841,7 +973,7 @@
         <v>-121.641075</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -849,10 +981,10 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
         <v>14</v>
@@ -876,7 +1008,7 @@
         <v>-121.640055</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -884,10 +1016,10 @@
         <v>11</v>
       </c>
       <c r="C9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" t="s">
         <v>49</v>
-      </c>
-      <c r="D9" t="s">
-        <v>51</v>
       </c>
       <c r="E9" t="s">
         <v>14</v>
@@ -911,7 +1043,7 @@
         <v>-121.639974</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -919,10 +1051,10 @@
         <v>11</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E10" t="s">
         <v>14</v>
@@ -946,7 +1078,7 @@
         <v>-121.672147</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -981,7 +1113,7 @@
         <v>-121.64358</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -989,7 +1121,7 @@
         <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
         <v>26</v>
@@ -1016,7 +1148,7 @@
         <v>-121.655367</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1024,16 +1156,16 @@
         <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E13" t="s">
         <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G13" t="s">
         <v>16</v>
@@ -1051,7 +1183,7 @@
         <v>-121.63758900000001</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1059,10 +1191,10 @@
         <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E14" t="s">
         <v>19</v>
@@ -1086,7 +1218,7 @@
         <v>-121.605636</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1094,10 +1226,10 @@
         <v>25</v>
       </c>
       <c r="C15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" t="s">
         <v>38</v>
-      </c>
-      <c r="D15" t="s">
-        <v>39</v>
       </c>
       <c r="E15" t="s">
         <v>19</v>
@@ -1121,7 +1253,7 @@
         <v>-121.572649</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1129,19 +1261,19 @@
         <v>25</v>
       </c>
       <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
         <v>46</v>
-      </c>
-      <c r="D16" t="s">
-        <v>48</v>
       </c>
       <c r="E16" t="s">
         <v>14</v>
       </c>
       <c r="F16" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G16" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H16" t="s">
         <v>16</v>
@@ -1156,7 +1288,7 @@
         <v>-121.587768</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1164,10 +1296,10 @@
         <v>25</v>
       </c>
       <c r="C17" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D17" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E17" t="s">
         <v>14</v>
@@ -1191,7 +1323,7 @@
         <v>-121.582909</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1199,10 +1331,10 @@
         <v>25</v>
       </c>
       <c r="C18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D18" t="s">
-        <v>27</v>
+        <v>68</v>
       </c>
       <c r="E18" t="s">
         <v>14</v>
@@ -1226,18 +1358,18 @@
         <v>-121.58289499999999</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="D19" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E19" t="s">
         <v>14</v>
@@ -1246,168 +1378,285 @@
         <v>15</v>
       </c>
       <c r="G19" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H19" t="s">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="I19" t="s">
         <v>16</v>
       </c>
       <c r="J19">
-        <v>38.476303000000001</v>
+        <v>38.544499999999999</v>
       </c>
       <c r="K19">
-        <v>-121.58860199999999</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+        <v>-121.58663900000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" t="s">
+        <v>15</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" t="s">
+        <v>56</v>
+      </c>
+      <c r="I20" t="s">
+        <v>16</v>
+      </c>
+      <c r="J20">
+        <v>38.476303000000001</v>
+      </c>
+      <c r="K20">
+        <v>-121.58860199999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" t="s">
         <v>28</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D21" t="s">
         <v>29</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E21" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" t="s">
+        <v>15</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" t="s">
+        <v>15</v>
+      </c>
+      <c r="J21">
+        <v>38.389926000000003</v>
+      </c>
+      <c r="K21">
+        <v>-121.628434</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" t="s">
+        <v>61</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" t="s">
+        <v>16</v>
+      </c>
+      <c r="H22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" t="s">
+        <v>16</v>
+      </c>
+      <c r="J22">
+        <v>38.390438000000003</v>
+      </c>
+      <c r="K22">
+        <v>-121.626563</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" t="s">
         <v>30</v>
       </c>
-      <c r="E20" t="s">
-        <v>19</v>
-      </c>
-      <c r="F20" t="s">
-        <v>15</v>
-      </c>
-      <c r="G20" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" t="s">
-        <v>15</v>
-      </c>
-      <c r="I20" t="s">
-        <v>15</v>
-      </c>
-      <c r="J20">
-        <v>38.389926000000003</v>
-      </c>
-      <c r="K20">
-        <v>-121.628434</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B21" t="s">
-        <v>28</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D23" t="s">
+        <v>31</v>
+      </c>
+      <c r="E23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" t="s">
+        <v>15</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" t="s">
+        <v>15</v>
+      </c>
+      <c r="J23">
+        <v>38.418415000000003</v>
+      </c>
+      <c r="K23">
+        <v>-121.615256</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" t="s">
+        <v>32</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="s">
+        <v>15</v>
+      </c>
+      <c r="I24" t="s">
+        <v>16</v>
+      </c>
+      <c r="J24">
+        <v>38.353357000000003</v>
+      </c>
+      <c r="K24">
+        <v>-121.643249</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25" t="s">
         <v>64</v>
       </c>
-      <c r="D21" t="s">
-        <v>63</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="E25" t="s">
         <v>14</v>
       </c>
-      <c r="F21" t="s">
-        <v>15</v>
-      </c>
-      <c r="G21" t="s">
-        <v>16</v>
-      </c>
-      <c r="H21" t="s">
-        <v>15</v>
-      </c>
-      <c r="I21" t="s">
-        <v>16</v>
-      </c>
-      <c r="J21">
-        <v>38.390438000000003</v>
-      </c>
-      <c r="K21">
-        <v>-121.626563</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A22">
-        <v>20</v>
-      </c>
-      <c r="B22" t="s">
-        <v>28</v>
-      </c>
-      <c r="C22" t="s">
-        <v>31</v>
-      </c>
-      <c r="D22" t="s">
-        <v>32</v>
-      </c>
-      <c r="E22" t="s">
-        <v>22</v>
-      </c>
-      <c r="F22" t="s">
-        <v>15</v>
-      </c>
-      <c r="G22" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" t="s">
-        <v>15</v>
-      </c>
-      <c r="I22" t="s">
-        <v>15</v>
-      </c>
-      <c r="J22">
-        <v>38.418415000000003</v>
-      </c>
-      <c r="K22">
-        <v>-121.615256</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A23">
-        <v>21</v>
-      </c>
-      <c r="B23" t="s">
-        <v>28</v>
-      </c>
-      <c r="C23" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" t="s">
-        <v>33</v>
-      </c>
-      <c r="E23" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" t="s">
-        <v>15</v>
-      </c>
-      <c r="G23" t="s">
-        <v>15</v>
-      </c>
-      <c r="H23" t="s">
-        <v>15</v>
-      </c>
-      <c r="I23" t="s">
-        <v>16</v>
-      </c>
-      <c r="J23">
-        <v>38.353357000000003</v>
-      </c>
-      <c r="K23">
-        <v>-121.643249</v>
+      <c r="F25" t="s">
+        <v>15</v>
+      </c>
+      <c r="G25" t="s">
+        <v>16</v>
+      </c>
+      <c r="H25" t="s">
+        <v>15</v>
+      </c>
+      <c r="I25" t="s">
+        <v>16</v>
+      </c>
+      <c r="J25">
+        <v>38.274275000000003</v>
+      </c>
+      <c r="K25">
+        <v>-121.66417800000001</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:I23">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="p">
+  <conditionalFormatting sqref="F2:I18 F20:I25">
+    <cfRule type="containsText" dxfId="14" priority="13" operator="containsText" text="p">
       <formula>NOT(ISERROR(SEARCH("p",F2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="y">
+    <cfRule type="containsText" dxfId="13" priority="14" operator="containsText" text="y">
       <formula>NOT(ISERROR(SEARCH("y",F2)))</formula>
     </cfRule>
+    <cfRule type="containsText" dxfId="12" priority="15" operator="containsText" text="n">
+      <formula>NOT(ISERROR(SEARCH("n",F2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H19">
+    <cfRule type="containsText" dxfId="11" priority="10" operator="containsText" text="p">
+      <formula>NOT(ISERROR(SEARCH("p",H19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="y">
+      <formula>NOT(ISERROR(SEARCH("y",H19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="n">
+      <formula>NOT(ISERROR(SEARCH("n",H19)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I19">
+    <cfRule type="containsText" dxfId="8" priority="7" operator="containsText" text="p">
+      <formula>NOT(ISERROR(SEARCH("p",I19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="y">
+      <formula>NOT(ISERROR(SEARCH("y",I19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="6" priority="9" operator="containsText" text="n">
+      <formula>NOT(ISERROR(SEARCH("n",I19)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19">
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="p">
+      <formula>NOT(ISERROR(SEARCH("p",G19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="y">
+      <formula>NOT(ISERROR(SEARCH("y",G19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="n">
+      <formula>NOT(ISERROR(SEARCH("n",G19)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F19">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="p">
+      <formula>NOT(ISERROR(SEARCH("p",F19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="y">
+      <formula>NOT(ISERROR(SEARCH("y",F19)))</formula>
+    </cfRule>
     <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="n">
-      <formula>NOT(ISERROR(SEARCH("n",F2)))</formula>
+      <formula>NOT(ISERROR(SEARCH("n",F19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
random updates, PCA for poster
</commit_message>
<xml_diff>
--- a/Data/tabular/YBLTE_sites.xlsx
+++ b/Data/tabular/YBLTE_sites.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kristinn\Downloads\coding\YBLTE\Data\tabular\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E47CBBAC-6BA7-406A-B016-AB1330D7E8DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA344C9-C51B-4B1B-B372-C35AA8D4757E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -302,97 +302,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFD5D5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFCD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFD5D5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFCD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFD5D5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFCD"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -1382,7 +1292,7 @@
         <v>15</v>
       </c>
       <c r="G18" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H18" t="s">
         <v>16</v>
@@ -1587,7 +1497,7 @@
         <v>-121.626563</v>
       </c>
       <c r="L23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
@@ -1705,48 +1615,15 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:I14 F16:I26">
-    <cfRule type="containsText" dxfId="11" priority="10" operator="containsText" text="p">
+  <conditionalFormatting sqref="F2:I26">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="p">
       <formula>NOT(ISERROR(SEARCH("p",F2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="11" operator="containsText" text="y">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="y">
       <formula>NOT(ISERROR(SEARCH("y",F2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="12" operator="containsText" text="n">
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="n">
       <formula>NOT(ISERROR(SEARCH("n",F2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F15 H15">
-    <cfRule type="containsText" dxfId="8" priority="7" operator="containsText" text="p">
-      <formula>NOT(ISERROR(SEARCH("p",F15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="y">
-      <formula>NOT(ISERROR(SEARCH("y",F15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="9" operator="containsText" text="n">
-      <formula>NOT(ISERROR(SEARCH("n",F15)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G15">
-    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="p">
-      <formula>NOT(ISERROR(SEARCH("p",G15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="y">
-      <formula>NOT(ISERROR(SEARCH("y",G15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="n">
-      <formula>NOT(ISERROR(SEARCH("n",G15)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I15">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="p">
-      <formula>NOT(ISERROR(SEARCH("p",I15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="y">
-      <formula>NOT(ISERROR(SEARCH("y",I15)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="n">
-      <formula>NOT(ISERROR(SEARCH("n",I15)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>